<commit_message>
Finished first question in optical flow
</commit_message>
<xml_diff>
--- a/computer_vision/course schedule.xlsx
+++ b/computer_vision/course schedule.xlsx
@@ -1,26 +1,39 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27726"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="5" rupBuild="27830"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ron Tohar\Desktop\הכשרה\CV_training\computer_vision\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{51C74C8F-56F1-4544-A2C6-CD119577D0F3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{DE2D0081-36B2-40E1-9F14-1359C78B7783}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14595" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="2062" yWindow="2835" windowWidth="16876" windowHeight="10418" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="227">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="228">
   <si>
     <t>Unit</t>
   </si>
@@ -701,6 +714,9 @@
   </si>
   <si>
     <t>Final Exam (T-Square)</t>
+  </si>
+  <si>
+    <t>74 - 7:30</t>
   </si>
 </sst>
 </file>
@@ -1902,7 +1918,9 @@
       </c>
       <c r="H35" s="6"/>
       <c r="J35" s="3"/>
-      <c r="L35" s="6"/>
+      <c r="L35" s="6">
+        <v>62</v>
+      </c>
     </row>
     <row r="36" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
@@ -2030,7 +2048,9 @@
       </c>
       <c r="H42" s="6"/>
       <c r="J42" s="3"/>
-      <c r="L42" s="6"/>
+      <c r="L42" s="6" t="s">
+        <v>227</v>
+      </c>
     </row>
     <row r="43" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" t="s">

</xml_diff>

<commit_message>
finished all 6 assignments
</commit_message>
<xml_diff>
--- a/computer_vision/course schedule.xlsx
+++ b/computer_vision/course schedule.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Ron Tohar\Desktop\הכשרה\CV_training\computer_vision\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AA68CBC8-8776-4F4C-9678-9C0EEC6A52AA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7AFBA225-E65D-4F52-8AEE-F8126A98E6D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2400" yWindow="3173" windowWidth="16875" windowHeight="10417" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-98" yWindow="-98" windowWidth="22695" windowHeight="14595" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="245" uniqueCount="228">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="242" uniqueCount="225">
   <si>
     <t>Unit</t>
   </si>
@@ -65,9 +65,6 @@
     <t>exact time</t>
   </si>
   <si>
-    <t>Column1</t>
-  </si>
-  <si>
     <t>yael vid#</t>
   </si>
   <si>
@@ -143,9 +140,6 @@
     <t>15/127</t>
   </si>
   <si>
-    <t>בתכלס מדבר על זה בעיקר בסרטון אחרי זה (15) בדקה 5:40</t>
-  </si>
-  <si>
     <t>2B</t>
   </si>
   <si>
@@ -165,9 +159,6 @@
   </si>
   <si>
     <t>17/127</t>
-  </si>
-  <si>
-    <t>מתחיל מסוף סרטון קודם הסברים אבל המילה hough transform מופיעה איפה שכתבתי פעם ראשונה</t>
   </si>
   <si>
     <t>2B-L2</t>
@@ -824,9 +815,9 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:L70" totalsRowShown="0">
-  <autoFilter ref="A1:L70" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
-  <tableColumns count="12">
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{00000000-000C-0000-FFFF-FFFF00000000}" name="Table1" displayName="Table1" ref="A1:K70" totalsRowShown="0">
+  <autoFilter ref="A1:K70" xr:uid="{00000000-0009-0000-0100-000001000000}"/>
+  <tableColumns count="11">
     <tableColumn id="1" xr3:uid="{00000000-0010-0000-0000-000001000000}" name="Unit"/>
     <tableColumn id="2" xr3:uid="{00000000-0010-0000-0000-000002000000}" name="Title"/>
     <tableColumn id="3" xr3:uid="{00000000-0010-0000-0000-000003000000}" name="Lesson"/>
@@ -837,7 +828,6 @@
     <tableColumn id="8" xr3:uid="{00000000-0010-0000-0000-000008000000}" name="# Video"/>
     <tableColumn id="9" xr3:uid="{00000000-0010-0000-0000-000009000000}" name="video number in playlist"/>
     <tableColumn id="10" xr3:uid="{00000000-0010-0000-0000-00000A000000}" name="exact time"/>
-    <tableColumn id="11" xr3:uid="{00000000-0010-0000-0000-00000B000000}" name="Column1"/>
     <tableColumn id="12" xr3:uid="{00000000-0010-0000-0000-00000C000000}" name="yael vid#"/>
   </tableColumns>
   <tableStyleInfo name="TableStyleLight1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
@@ -1132,7 +1122,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0"/>
   </sheetPr>
-  <dimension ref="A1:L70"/>
+  <dimension ref="A1:K70"/>
   <sheetFormatPr defaultRowHeight="13.5" x14ac:dyDescent="0.35"/>
   <cols>
     <col min="1" max="1" width="6.75" bestFit="1" customWidth="1"/>
@@ -1145,11 +1135,10 @@
     <col min="8" max="8" width="9" style="9" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="13.5625" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="13.5625" style="10" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="13.5625" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="12" style="9" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="12" style="9" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="1" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -1180,53 +1169,50 @@
       <c r="J1" s="3" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+    </row>
+    <row r="2" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A2" t="s">
         <v>11</v>
       </c>
-    </row>
-    <row r="2" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A2" t="s">
+      <c r="B2" t="s">
         <v>12</v>
       </c>
-      <c r="B2" t="s">
+      <c r="C2" t="s">
         <v>13</v>
       </c>
-      <c r="C2" t="s">
-        <v>14</v>
-      </c>
       <c r="D2" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="E2" s="4">
         <v>42</v>
       </c>
       <c r="F2" s="5" t="s">
+        <v>14</v>
+      </c>
+      <c r="G2" t="s">
         <v>15</v>
-      </c>
-      <c r="G2" t="s">
-        <v>16</v>
       </c>
       <c r="H2" s="4">
         <v>1</v>
       </c>
       <c r="J2" s="3"/>
-      <c r="L2" s="6"/>
-    </row>
-    <row r="3" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K2" s="6"/>
+    </row>
+    <row r="3" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A3" t="s">
+        <v>16</v>
+      </c>
+      <c r="B3" t="s">
         <v>17</v>
       </c>
-      <c r="B3" t="s">
+      <c r="C3" t="s">
         <v>18</v>
       </c>
-      <c r="C3" t="s">
+      <c r="D3" t="s">
         <v>19</v>
-      </c>
-      <c r="D3" t="s">
-        <v>20</v>
       </c>
       <c r="E3" s="4">
         <v>44</v>
@@ -1235,14 +1221,14 @@
         <v>2</v>
       </c>
       <c r="J3" s="3"/>
-      <c r="L3" s="6"/>
-    </row>
-    <row r="4" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K3" s="6"/>
+    </row>
+    <row r="4" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C4" t="s">
+        <v>20</v>
+      </c>
+      <c r="D4" t="s">
         <v>21</v>
-      </c>
-      <c r="D4" t="s">
-        <v>22</v>
       </c>
       <c r="E4" s="4">
         <v>24</v>
@@ -1251,17 +1237,17 @@
         <v>7.5</v>
       </c>
       <c r="I4" t="s">
+        <v>22</v>
+      </c>
+      <c r="J4" s="3"/>
+      <c r="K4" s="6"/>
+    </row>
+    <row r="5" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C5" t="s">
         <v>23</v>
       </c>
-      <c r="J4" s="3"/>
-      <c r="L4" s="6"/>
-    </row>
-    <row r="5" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C5" t="s">
+      <c r="D5" t="s">
         <v>24</v>
-      </c>
-      <c r="D5" t="s">
-        <v>25</v>
       </c>
       <c r="E5" s="4">
         <v>34</v>
@@ -1270,17 +1256,17 @@
         <v>8</v>
       </c>
       <c r="I5" t="s">
+        <v>25</v>
+      </c>
+      <c r="J5" s="3"/>
+      <c r="K5" s="6"/>
+    </row>
+    <row r="6" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C6" t="s">
         <v>26</v>
       </c>
-      <c r="J5" s="3"/>
-      <c r="L5" s="6"/>
-    </row>
-    <row r="6" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C6" t="s">
+      <c r="D6" t="s">
         <v>27</v>
-      </c>
-      <c r="D6" t="s">
-        <v>28</v>
       </c>
       <c r="E6" s="4">
         <v>13</v>
@@ -1289,19 +1275,19 @@
         <v>11</v>
       </c>
       <c r="I6" s="2" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="J6" s="8">
         <v>2.2768518518518519</v>
       </c>
-      <c r="L6" s="6"/>
-    </row>
-    <row r="7" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K6" s="6"/>
+    </row>
+    <row r="7" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C7" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" t="s">
         <v>30</v>
-      </c>
-      <c r="D7" t="s">
-        <v>31</v>
       </c>
       <c r="E7" s="4">
         <v>27</v>
@@ -1310,17 +1296,17 @@
         <v>12</v>
       </c>
       <c r="I7" t="s">
+        <v>31</v>
+      </c>
+      <c r="J7" s="3"/>
+      <c r="K7" s="6"/>
+    </row>
+    <row r="8" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="C8" t="s">
         <v>32</v>
       </c>
-      <c r="J7" s="3"/>
-      <c r="L7" s="6"/>
-    </row>
-    <row r="8" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="C8" t="s">
+      <c r="D8" t="s">
         <v>33</v>
-      </c>
-      <c r="D8" t="s">
-        <v>34</v>
       </c>
       <c r="E8" s="4">
         <v>19</v>
@@ -1329,58 +1315,52 @@
         <v>14</v>
       </c>
       <c r="I8" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="J8" s="8">
         <v>2.2525462962962965</v>
       </c>
-      <c r="K8" t="s">
+      <c r="K8" s="6"/>
+    </row>
+    <row r="9" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A9" t="s">
+        <v>35</v>
+      </c>
+      <c r="B9" t="s">
         <v>36</v>
       </c>
-      <c r="L8" s="6"/>
-    </row>
-    <row r="9" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A9" t="s">
+      <c r="C9" t="s">
         <v>37</v>
       </c>
-      <c r="B9" t="s">
+      <c r="D9" t="s">
         <v>38</v>
-      </c>
-      <c r="C9" t="s">
-        <v>39</v>
-      </c>
-      <c r="D9" t="s">
-        <v>40</v>
       </c>
       <c r="E9" s="4">
         <v>36</v>
       </c>
       <c r="F9" s="5" t="s">
-        <v>41</v>
+        <v>39</v>
       </c>
       <c r="G9" t="s">
-        <v>42</v>
+        <v>40</v>
       </c>
       <c r="H9" s="4">
         <v>16</v>
       </c>
       <c r="I9" t="s">
-        <v>43</v>
+        <v>41</v>
       </c>
       <c r="J9" s="8">
         <v>2.2074074074074073</v>
       </c>
-      <c r="K9" t="s">
-        <v>44</v>
-      </c>
-      <c r="L9" s="6"/>
-    </row>
-    <row r="10" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K9" s="6"/>
+    </row>
+    <row r="10" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C10" t="s">
-        <v>45</v>
+        <v>42</v>
       </c>
       <c r="D10" t="s">
-        <v>46</v>
+        <v>43</v>
       </c>
       <c r="E10" s="4">
         <v>13</v>
@@ -1389,19 +1369,19 @@
         <v>18</v>
       </c>
       <c r="I10" t="s">
-        <v>47</v>
+        <v>44</v>
       </c>
       <c r="J10" s="8">
         <v>2.1310185185185184</v>
       </c>
-      <c r="L10" s="6"/>
-    </row>
-    <row r="11" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K10" s="6"/>
+    </row>
+    <row r="11" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C11" t="s">
-        <v>48</v>
+        <v>45</v>
       </c>
       <c r="D11" t="s">
-        <v>49</v>
+        <v>46</v>
       </c>
       <c r="E11" s="4">
         <v>16</v>
@@ -1410,25 +1390,25 @@
         <v>19</v>
       </c>
       <c r="I11" t="s">
-        <v>50</v>
+        <v>47</v>
       </c>
       <c r="J11" s="8">
         <v>2.0268518518518519</v>
       </c>
-      <c r="L11" s="6"/>
-    </row>
-    <row r="12" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K11" s="6"/>
+    </row>
+    <row r="12" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A12" t="s">
+        <v>48</v>
+      </c>
+      <c r="B12" t="s">
+        <v>49</v>
+      </c>
+      <c r="C12" t="s">
+        <v>50</v>
+      </c>
+      <c r="D12" t="s">
         <v>51</v>
-      </c>
-      <c r="B12" t="s">
-        <v>52</v>
-      </c>
-      <c r="C12" t="s">
-        <v>53</v>
-      </c>
-      <c r="D12" t="s">
-        <v>54</v>
       </c>
       <c r="E12" s="4">
         <v>36</v>
@@ -1437,19 +1417,19 @@
         <v>20</v>
       </c>
       <c r="I12" t="s">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="J12" s="3"/>
-      <c r="L12" s="4">
+      <c r="K12" s="4">
         <v>21</v>
       </c>
     </row>
-    <row r="13" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="13" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C13" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="D13" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="E13" s="4">
         <v>22</v>
@@ -1458,19 +1438,19 @@
         <v>22</v>
       </c>
       <c r="I13" t="s">
-        <v>58</v>
+        <v>55</v>
       </c>
       <c r="J13" s="3"/>
-      <c r="L13" s="4">
+      <c r="K13" s="4">
         <v>22</v>
       </c>
     </row>
-    <row r="14" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="14" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C14" t="s">
-        <v>59</v>
+        <v>56</v>
       </c>
       <c r="D14" t="s">
-        <v>60</v>
+        <v>57</v>
       </c>
       <c r="E14" s="4">
         <v>35</v>
@@ -1479,27 +1459,27 @@
         <v>23</v>
       </c>
       <c r="I14" t="s">
-        <v>61</v>
+        <v>58</v>
       </c>
       <c r="J14" s="8">
         <v>2.5025462962962965</v>
       </c>
-      <c r="L14" s="4">
+      <c r="K14" s="4">
         <v>24</v>
       </c>
     </row>
-    <row r="15" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="15" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A15" t="s">
+        <v>59</v>
+      </c>
+      <c r="B15" t="s">
+        <v>60</v>
+      </c>
+      <c r="C15" t="s">
+        <v>61</v>
+      </c>
+      <c r="D15" t="s">
         <v>62</v>
-      </c>
-      <c r="B15" t="s">
-        <v>63</v>
-      </c>
-      <c r="C15" t="s">
-        <v>64</v>
-      </c>
-      <c r="D15" t="s">
-        <v>65</v>
       </c>
       <c r="E15" s="4">
         <v>33</v>
@@ -1508,57 +1488,57 @@
         <v>26</v>
       </c>
       <c r="I15" t="s">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="J15" s="3"/>
-      <c r="L15" s="4">
+      <c r="K15" s="4">
         <v>27</v>
       </c>
     </row>
-    <row r="16" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="16" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C16" t="s">
-        <v>67</v>
+        <v>64</v>
       </c>
       <c r="D16" t="s">
-        <v>68</v>
+        <v>65</v>
       </c>
       <c r="E16" s="4">
         <v>26</v>
       </c>
       <c r="H16" s="6"/>
       <c r="J16" s="3"/>
-      <c r="L16" s="4">
+      <c r="K16" s="4">
         <v>29</v>
       </c>
     </row>
-    <row r="17" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="17" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A17" t="s">
-        <v>69</v>
+        <v>66</v>
       </c>
       <c r="B17" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="C17" t="s">
-        <v>71</v>
+        <v>68</v>
       </c>
       <c r="D17" t="s">
-        <v>70</v>
+        <v>67</v>
       </c>
       <c r="E17" s="4">
         <v>26</v>
       </c>
       <c r="H17" s="6"/>
       <c r="J17" s="3"/>
-      <c r="L17" s="4">
+      <c r="K17" s="4">
         <v>31</v>
       </c>
     </row>
-    <row r="18" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="18" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C18" t="s">
-        <v>72</v>
+        <v>69</v>
       </c>
       <c r="D18" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="E18" s="4">
         <v>11</v>
@@ -1567,54 +1547,54 @@
         <v>32</v>
       </c>
       <c r="I18" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="J18" s="8"/>
-      <c r="L18" s="4">
+      <c r="K18" s="4">
         <v>33</v>
       </c>
     </row>
-    <row r="19" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="19" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C19" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="D19" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="E19" s="4">
         <v>29</v>
       </c>
       <c r="F19" s="5" t="s">
-        <v>77</v>
+        <v>74</v>
       </c>
       <c r="G19" t="s">
-        <v>78</v>
+        <v>75</v>
       </c>
       <c r="H19" s="4">
         <v>32</v>
       </c>
       <c r="I19" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="J19" s="8">
         <v>2.5407407407407407</v>
       </c>
-      <c r="L19" s="4">
+      <c r="K19" s="4">
         <v>33</v>
       </c>
     </row>
-    <row r="20" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="20" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A20" t="s">
+        <v>76</v>
+      </c>
+      <c r="B20" t="s">
+        <v>77</v>
+      </c>
+      <c r="C20" t="s">
+        <v>78</v>
+      </c>
+      <c r="D20" t="s">
         <v>79</v>
-      </c>
-      <c r="B20" t="s">
-        <v>80</v>
-      </c>
-      <c r="C20" t="s">
-        <v>81</v>
-      </c>
-      <c r="D20" t="s">
-        <v>82</v>
       </c>
       <c r="E20" s="4">
         <v>24</v>
@@ -1623,915 +1603,915 @@
         <v>35</v>
       </c>
       <c r="I20" t="s">
-        <v>83</v>
+        <v>80</v>
       </c>
       <c r="J20" s="3"/>
-      <c r="L20" s="4">
+      <c r="K20" s="4">
         <v>36</v>
       </c>
     </row>
-    <row r="21" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="21" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C21" t="s">
-        <v>84</v>
+        <v>81</v>
       </c>
       <c r="D21" t="s">
-        <v>85</v>
+        <v>82</v>
       </c>
       <c r="E21" s="4">
         <v>16</v>
       </c>
       <c r="H21" s="6"/>
       <c r="J21" s="3"/>
-      <c r="L21" s="4">
+      <c r="K21" s="4">
         <v>37</v>
       </c>
     </row>
-    <row r="22" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="22" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C22" t="s">
-        <v>86</v>
+        <v>83</v>
       </c>
       <c r="D22" t="s">
-        <v>87</v>
+        <v>84</v>
       </c>
       <c r="E22" s="4">
         <v>31</v>
       </c>
       <c r="H22" s="6"/>
       <c r="J22" s="3"/>
-      <c r="L22" s="4">
+      <c r="K22" s="4">
         <v>41</v>
       </c>
     </row>
-    <row r="23" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="23" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A23" t="s">
+        <v>85</v>
+      </c>
+      <c r="B23" t="s">
+        <v>86</v>
+      </c>
+      <c r="C23" t="s">
+        <v>87</v>
+      </c>
+      <c r="D23" t="s">
         <v>88</v>
-      </c>
-      <c r="B23" t="s">
-        <v>89</v>
-      </c>
-      <c r="C23" t="s">
-        <v>90</v>
-      </c>
-      <c r="D23" t="s">
-        <v>91</v>
       </c>
       <c r="E23" s="4">
         <v>10</v>
       </c>
       <c r="F23" s="5" t="s">
+        <v>89</v>
+      </c>
+      <c r="G23" t="s">
+        <v>90</v>
+      </c>
+      <c r="H23" s="1" t="s">
+        <v>91</v>
+      </c>
+      <c r="I23" t="s">
         <v>92</v>
-      </c>
-      <c r="G23" t="s">
-        <v>93</v>
-      </c>
-      <c r="H23" s="1" t="s">
-        <v>94</v>
-      </c>
-      <c r="I23" t="s">
-        <v>95</v>
       </c>
       <c r="J23" s="8">
         <v>2.0199074074074073</v>
       </c>
-      <c r="L23" s="4">
+      <c r="K23" s="4">
         <v>42</v>
       </c>
     </row>
-    <row r="24" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="24" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C24" t="s">
-        <v>96</v>
+        <v>93</v>
       </c>
       <c r="D24" t="s">
-        <v>97</v>
+        <v>94</v>
       </c>
       <c r="E24" s="4">
         <v>33</v>
       </c>
       <c r="H24" s="6"/>
       <c r="I24" t="s">
-        <v>95</v>
+        <v>92</v>
       </c>
       <c r="J24" s="8">
         <v>2.5407407407407407</v>
       </c>
-      <c r="L24" s="7">
+      <c r="K24" s="7">
         <v>42.9</v>
       </c>
     </row>
-    <row r="25" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="25" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C25" t="s">
-        <v>98</v>
+        <v>95</v>
       </c>
       <c r="D25" t="s">
-        <v>99</v>
+        <v>96</v>
       </c>
       <c r="E25" s="4">
         <v>14</v>
       </c>
       <c r="H25" s="6"/>
       <c r="J25" s="3"/>
-      <c r="L25" s="4">
+      <c r="K25" s="4">
         <v>45</v>
       </c>
     </row>
-    <row r="26" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="26" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C26" t="s">
-        <v>100</v>
+        <v>97</v>
       </c>
       <c r="D26" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="E26" s="4">
         <v>22</v>
       </c>
       <c r="H26" s="6"/>
       <c r="J26" s="3"/>
-      <c r="L26" s="4">
+      <c r="K26" s="4">
         <v>46</v>
       </c>
     </row>
-    <row r="27" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="27" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C27" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
       <c r="D27" t="s">
-        <v>103</v>
+        <v>100</v>
       </c>
       <c r="E27" s="4">
         <v>37</v>
       </c>
       <c r="H27" s="6"/>
       <c r="J27" s="3"/>
-      <c r="L27" s="7">
+      <c r="K27" s="7">
         <v>47.5</v>
       </c>
     </row>
-    <row r="28" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="28" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A28" t="s">
+        <v>101</v>
+      </c>
+      <c r="B28" t="s">
+        <v>102</v>
+      </c>
+      <c r="C28" t="s">
+        <v>103</v>
+      </c>
+      <c r="D28" t="s">
         <v>104</v>
-      </c>
-      <c r="B28" t="s">
-        <v>105</v>
-      </c>
-      <c r="C28" t="s">
-        <v>106</v>
-      </c>
-      <c r="D28" t="s">
-        <v>107</v>
       </c>
       <c r="E28" s="4">
         <v>13</v>
       </c>
       <c r="F28" s="5" t="s">
-        <v>108</v>
+        <v>105</v>
       </c>
       <c r="G28" t="s">
-        <v>109</v>
+        <v>106</v>
       </c>
       <c r="H28" s="6"/>
       <c r="J28" s="3"/>
-      <c r="L28" s="4">
+      <c r="K28" s="4">
         <v>50</v>
       </c>
     </row>
-    <row r="29" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="29" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C29" t="s">
-        <v>110</v>
+        <v>107</v>
       </c>
       <c r="D29" t="s">
-        <v>111</v>
+        <v>108</v>
       </c>
       <c r="E29" s="4">
         <v>39</v>
       </c>
       <c r="H29" s="6"/>
       <c r="J29" s="3"/>
-      <c r="L29" s="4">
+      <c r="K29" s="4">
         <v>51</v>
       </c>
     </row>
-    <row r="30" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="30" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C30" t="s">
-        <v>112</v>
+        <v>109</v>
       </c>
       <c r="D30" t="s">
-        <v>113</v>
+        <v>110</v>
       </c>
       <c r="E30" s="4">
         <v>23</v>
       </c>
       <c r="H30" s="6"/>
       <c r="J30" s="3"/>
-      <c r="L30" s="1" t="s">
+      <c r="K30" s="1" t="s">
+        <v>111</v>
+      </c>
+    </row>
+    <row r="31" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="A31" t="s">
+        <v>112</v>
+      </c>
+      <c r="B31" t="s">
+        <v>113</v>
+      </c>
+      <c r="C31" t="s">
         <v>114</v>
       </c>
-    </row>
-    <row r="31" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
-      <c r="A31" t="s">
+      <c r="D31" t="s">
         <v>115</v>
-      </c>
-      <c r="B31" t="s">
-        <v>116</v>
-      </c>
-      <c r="C31" t="s">
-        <v>117</v>
-      </c>
-      <c r="D31" t="s">
-        <v>118</v>
       </c>
       <c r="E31" s="4">
         <v>27</v>
       </c>
       <c r="H31" s="6"/>
       <c r="J31" s="3"/>
-      <c r="L31" s="7">
+      <c r="K31" s="7">
         <v>54.5</v>
       </c>
     </row>
-    <row r="32" spans="1:12" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="32" spans="1:11" ht="20.25" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C32" t="s">
-        <v>119</v>
+        <v>116</v>
       </c>
       <c r="D32" t="s">
-        <v>120</v>
+        <v>117</v>
       </c>
       <c r="E32" s="4">
         <v>16</v>
       </c>
       <c r="H32" s="6"/>
       <c r="J32" s="3"/>
-      <c r="L32" s="4">
+      <c r="K32" s="4">
         <v>55</v>
       </c>
     </row>
-    <row r="33" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="33" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A33" t="s">
-        <v>121</v>
+        <v>118</v>
       </c>
       <c r="B33" t="s">
-        <v>38</v>
+        <v>36</v>
       </c>
       <c r="C33" t="s">
-        <v>122</v>
+        <v>119</v>
       </c>
       <c r="D33" t="s">
-        <v>123</v>
+        <v>120</v>
       </c>
       <c r="E33" s="4">
         <v>31</v>
       </c>
       <c r="H33" s="6"/>
       <c r="J33" s="3"/>
-      <c r="L33" s="6"/>
-    </row>
-    <row r="34" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K33" s="6"/>
+    </row>
+    <row r="34" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C34" t="s">
-        <v>124</v>
+        <v>121</v>
       </c>
       <c r="D34" t="s">
-        <v>125</v>
+        <v>122</v>
       </c>
       <c r="E34" s="4">
         <v>33</v>
       </c>
       <c r="H34" s="6"/>
       <c r="J34" s="3"/>
-      <c r="L34" s="4">
+      <c r="K34" s="4">
         <v>60</v>
       </c>
     </row>
-    <row r="35" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="35" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A35" t="s">
-        <v>126</v>
+        <v>123</v>
       </c>
       <c r="B35" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="C35" t="s">
-        <v>128</v>
+        <v>125</v>
       </c>
       <c r="D35" t="s">
-        <v>127</v>
+        <v>124</v>
       </c>
       <c r="E35" s="4">
         <v>35</v>
       </c>
       <c r="H35" s="6"/>
       <c r="J35" s="3"/>
-      <c r="L35" s="6">
+      <c r="K35" s="6">
         <v>62</v>
       </c>
     </row>
-    <row r="36" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="36" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A36" t="s">
-        <v>129</v>
+        <v>126</v>
       </c>
       <c r="B36" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="C36" t="s">
-        <v>131</v>
+        <v>128</v>
       </c>
       <c r="D36" t="s">
-        <v>130</v>
+        <v>127</v>
       </c>
       <c r="E36" s="4">
         <v>26</v>
       </c>
       <c r="H36" s="6"/>
       <c r="J36" s="3"/>
-      <c r="L36" s="6"/>
-    </row>
-    <row r="37" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K36" s="6"/>
+    </row>
+    <row r="37" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A37" t="s">
-        <v>132</v>
+        <v>129</v>
       </c>
       <c r="B37" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="C37" t="s">
-        <v>134</v>
+        <v>131</v>
       </c>
       <c r="D37" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E37" s="4">
         <v>34</v>
       </c>
       <c r="H37" s="6"/>
       <c r="J37" s="3"/>
-      <c r="L37" s="6"/>
-    </row>
-    <row r="38" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K37" s="6"/>
+    </row>
+    <row r="38" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A38" t="s">
+        <v>132</v>
+      </c>
+      <c r="B38" t="s">
+        <v>133</v>
+      </c>
+      <c r="C38" t="s">
+        <v>134</v>
+      </c>
+      <c r="D38" t="s">
         <v>135</v>
-      </c>
-      <c r="B38" t="s">
-        <v>136</v>
-      </c>
-      <c r="C38" t="s">
-        <v>137</v>
-      </c>
-      <c r="D38" t="s">
-        <v>138</v>
       </c>
       <c r="E38" s="4">
         <v>16</v>
       </c>
       <c r="F38" s="5" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="G38" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="H38" s="6"/>
       <c r="J38" s="3"/>
-      <c r="L38" s="6"/>
-    </row>
-    <row r="39" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K38" s="6"/>
+    </row>
+    <row r="39" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A39" t="s">
+        <v>138</v>
+      </c>
+      <c r="B39" t="s">
+        <v>139</v>
+      </c>
+      <c r="C39" t="s">
+        <v>140</v>
+      </c>
+      <c r="D39" t="s">
         <v>141</v>
-      </c>
-      <c r="B39" t="s">
-        <v>142</v>
-      </c>
-      <c r="C39" t="s">
-        <v>143</v>
-      </c>
-      <c r="D39" t="s">
-        <v>144</v>
       </c>
       <c r="E39" s="4">
         <v>24</v>
       </c>
       <c r="H39" s="6"/>
       <c r="J39" s="3"/>
-      <c r="L39" s="6"/>
-    </row>
-    <row r="40" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K39" s="6"/>
+    </row>
+    <row r="40" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C40" t="s">
-        <v>145</v>
+        <v>142</v>
       </c>
       <c r="D40" t="s">
-        <v>146</v>
+        <v>143</v>
       </c>
       <c r="E40" s="4">
         <v>17</v>
       </c>
       <c r="H40" s="6"/>
       <c r="J40" s="3"/>
-      <c r="L40" s="6"/>
-    </row>
-    <row r="41" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K40" s="6"/>
+    </row>
+    <row r="41" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C41" t="s">
-        <v>147</v>
+        <v>144</v>
       </c>
       <c r="D41" t="s">
-        <v>148</v>
+        <v>145</v>
       </c>
       <c r="E41" s="4">
         <v>33</v>
       </c>
       <c r="H41" s="6"/>
       <c r="J41" s="3"/>
-      <c r="L41" s="6"/>
-    </row>
-    <row r="42" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K41" s="6"/>
+    </row>
+    <row r="42" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C42" t="s">
-        <v>149</v>
+        <v>146</v>
       </c>
       <c r="D42" t="s">
-        <v>150</v>
+        <v>147</v>
       </c>
       <c r="E42" s="4">
         <v>24</v>
       </c>
       <c r="H42" s="6"/>
       <c r="J42" s="3"/>
-      <c r="L42" s="6" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="43" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K42" s="6" t="s">
+        <v>224</v>
+      </c>
+    </row>
+    <row r="43" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A43" t="s">
-        <v>151</v>
+        <v>148</v>
       </c>
       <c r="B43" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="C43" t="s">
-        <v>153</v>
+        <v>150</v>
       </c>
       <c r="D43" t="s">
-        <v>152</v>
+        <v>149</v>
       </c>
       <c r="E43" s="4">
         <v>14</v>
       </c>
       <c r="H43" s="6"/>
       <c r="J43" s="3"/>
-      <c r="L43" s="6"/>
-    </row>
-    <row r="44" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K43" s="6"/>
+    </row>
+    <row r="44" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A44" t="s">
+        <v>151</v>
+      </c>
+      <c r="B44" t="s">
+        <v>152</v>
+      </c>
+      <c r="C44" t="s">
+        <v>153</v>
+      </c>
+      <c r="D44" t="s">
         <v>154</v>
-      </c>
-      <c r="B44" t="s">
-        <v>155</v>
-      </c>
-      <c r="C44" t="s">
-        <v>156</v>
-      </c>
-      <c r="D44" t="s">
-        <v>157</v>
       </c>
       <c r="E44" s="4">
         <v>21</v>
       </c>
       <c r="H44" s="6"/>
       <c r="J44" s="3"/>
-      <c r="L44" s="6"/>
-    </row>
-    <row r="45" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K44" s="6"/>
+    </row>
+    <row r="45" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C45" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="D45" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="E45" s="4">
         <v>36</v>
       </c>
       <c r="H45" s="6"/>
       <c r="J45" s="3"/>
-      <c r="L45" s="6"/>
-    </row>
-    <row r="46" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K45" s="6"/>
+    </row>
+    <row r="46" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A46" t="s">
+        <v>157</v>
+      </c>
+      <c r="B46" t="s">
+        <v>158</v>
+      </c>
+      <c r="C46" t="s">
+        <v>159</v>
+      </c>
+      <c r="D46" t="s">
         <v>160</v>
-      </c>
-      <c r="B46" t="s">
-        <v>161</v>
-      </c>
-      <c r="C46" t="s">
-        <v>162</v>
-      </c>
-      <c r="D46" t="s">
-        <v>163</v>
       </c>
       <c r="E46" s="4">
         <v>23</v>
       </c>
       <c r="F46" s="5" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
       <c r="G46" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
       <c r="H46" s="6"/>
       <c r="J46" s="3"/>
-      <c r="L46" s="6">
+      <c r="K46" s="6">
         <v>83</v>
       </c>
     </row>
-    <row r="47" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="47" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C47" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
       <c r="D47" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
       <c r="E47" s="4">
         <v>17</v>
       </c>
       <c r="H47" s="6"/>
       <c r="J47" s="3"/>
-      <c r="L47" s="6"/>
-    </row>
-    <row r="48" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K47" s="6"/>
+    </row>
+    <row r="48" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C48" t="s">
-        <v>168</v>
+        <v>165</v>
       </c>
       <c r="D48" t="s">
-        <v>169</v>
+        <v>166</v>
       </c>
       <c r="E48" s="4">
         <v>24</v>
       </c>
       <c r="H48" s="6"/>
       <c r="J48" s="3"/>
-      <c r="L48" s="6"/>
-    </row>
-    <row r="49" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K48" s="6"/>
+    </row>
+    <row r="49" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C49" t="s">
-        <v>170</v>
+        <v>167</v>
       </c>
       <c r="D49" t="s">
-        <v>171</v>
+        <v>168</v>
       </c>
       <c r="E49" s="4">
         <v>15</v>
       </c>
       <c r="H49" s="6"/>
       <c r="J49" s="3"/>
-      <c r="L49" s="6"/>
-    </row>
-    <row r="50" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K49" s="6"/>
+    </row>
+    <row r="50" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A50" t="s">
-        <v>172</v>
+        <v>169</v>
       </c>
       <c r="B50" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="C50" t="s">
-        <v>174</v>
+        <v>171</v>
       </c>
       <c r="D50" t="s">
-        <v>173</v>
+        <v>170</v>
       </c>
       <c r="E50" s="4">
         <v>27</v>
       </c>
       <c r="H50" s="6"/>
       <c r="J50" s="3"/>
-      <c r="L50" s="6">
+      <c r="K50" s="6">
         <v>87</v>
       </c>
     </row>
-    <row r="51" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+    <row r="51" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A51" t="s">
-        <v>175</v>
+        <v>172</v>
       </c>
       <c r="B51" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="C51" t="s">
-        <v>177</v>
+        <v>174</v>
       </c>
       <c r="D51" t="s">
-        <v>176</v>
+        <v>173</v>
       </c>
       <c r="E51" s="4">
         <v>21</v>
       </c>
       <c r="H51" s="6"/>
       <c r="J51" s="3"/>
-      <c r="L51" s="6"/>
-    </row>
-    <row r="52" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K51" s="6"/>
+    </row>
+    <row r="52" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A52" t="s">
-        <v>178</v>
+        <v>175</v>
       </c>
       <c r="B52" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="C52" t="s">
-        <v>180</v>
+        <v>177</v>
       </c>
       <c r="D52" t="s">
-        <v>179</v>
+        <v>176</v>
       </c>
       <c r="E52" s="4">
         <v>28</v>
       </c>
       <c r="H52" s="6"/>
       <c r="J52" s="3"/>
-      <c r="L52" s="6"/>
-    </row>
-    <row r="53" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K52" s="6"/>
+    </row>
+    <row r="53" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C53" t="s">
-        <v>181</v>
+        <v>178</v>
       </c>
       <c r="D53" t="s">
-        <v>182</v>
+        <v>179</v>
       </c>
       <c r="E53" s="4">
         <v>48</v>
       </c>
       <c r="H53" s="6"/>
       <c r="J53" s="3"/>
-      <c r="L53" s="6"/>
-    </row>
-    <row r="54" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K53" s="6"/>
+    </row>
+    <row r="54" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C54" t="s">
-        <v>183</v>
+        <v>180</v>
       </c>
       <c r="D54" t="s">
-        <v>184</v>
+        <v>181</v>
       </c>
       <c r="E54" s="4">
         <v>26</v>
       </c>
       <c r="H54" s="6"/>
       <c r="J54" s="3"/>
-      <c r="L54" s="6"/>
-    </row>
-    <row r="55" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K54" s="6"/>
+    </row>
+    <row r="55" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A55" t="s">
-        <v>185</v>
+        <v>182</v>
       </c>
       <c r="B55" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="C55" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D55" t="s">
-        <v>186</v>
+        <v>183</v>
       </c>
       <c r="E55" s="4">
         <v>27</v>
       </c>
       <c r="H55" s="6"/>
       <c r="J55" s="3"/>
-      <c r="L55" s="6"/>
-    </row>
-    <row r="56" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K55" s="6"/>
+    </row>
+    <row r="56" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C56" t="s">
-        <v>188</v>
+        <v>185</v>
       </c>
       <c r="D56" t="s">
-        <v>189</v>
+        <v>186</v>
       </c>
       <c r="E56" s="4">
         <v>27</v>
       </c>
       <c r="H56" s="6"/>
       <c r="J56" s="3"/>
-      <c r="L56" s="6"/>
-    </row>
-    <row r="57" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K56" s="6"/>
+    </row>
+    <row r="57" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C57" t="s">
-        <v>190</v>
+        <v>187</v>
       </c>
       <c r="D57" t="s">
-        <v>191</v>
+        <v>188</v>
       </c>
       <c r="E57" s="4">
         <v>51</v>
       </c>
       <c r="H57" s="6"/>
       <c r="J57" s="3"/>
-      <c r="L57" s="6"/>
-    </row>
-    <row r="58" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K57" s="6"/>
+    </row>
+    <row r="58" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C58" t="s">
-        <v>192</v>
+        <v>189</v>
       </c>
       <c r="D58" t="s">
-        <v>193</v>
+        <v>190</v>
       </c>
       <c r="E58" s="4">
         <v>14</v>
       </c>
       <c r="H58" s="6"/>
       <c r="J58" s="3"/>
-      <c r="L58" s="6"/>
-    </row>
-    <row r="59" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K58" s="6"/>
+    </row>
+    <row r="59" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A59" t="s">
+        <v>191</v>
+      </c>
+      <c r="B59" t="s">
+        <v>192</v>
+      </c>
+      <c r="C59" t="s">
+        <v>193</v>
+      </c>
+      <c r="D59" t="s">
         <v>194</v>
-      </c>
-      <c r="B59" t="s">
-        <v>195</v>
-      </c>
-      <c r="C59" t="s">
-        <v>196</v>
-      </c>
-      <c r="D59" t="s">
-        <v>197</v>
       </c>
       <c r="E59" s="4">
         <v>24</v>
       </c>
       <c r="F59" t="s">
-        <v>198</v>
+        <v>195</v>
       </c>
       <c r="G59" t="s">
-        <v>199</v>
+        <v>196</v>
       </c>
       <c r="H59" s="6"/>
       <c r="J59" s="3"/>
-      <c r="L59" s="6"/>
-    </row>
-    <row r="60" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K59" s="6"/>
+    </row>
+    <row r="60" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C60" t="s">
-        <v>200</v>
+        <v>197</v>
       </c>
       <c r="D60" t="s">
-        <v>201</v>
+        <v>198</v>
       </c>
       <c r="E60" s="4">
         <v>32</v>
       </c>
       <c r="H60" s="6"/>
       <c r="J60" s="3"/>
-      <c r="L60" s="6"/>
-    </row>
-    <row r="61" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K60" s="6"/>
+    </row>
+    <row r="61" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C61" t="s">
-        <v>202</v>
+        <v>199</v>
       </c>
       <c r="D61" t="s">
-        <v>203</v>
+        <v>200</v>
       </c>
       <c r="E61" s="4">
         <v>46</v>
       </c>
       <c r="H61" s="6"/>
       <c r="J61" s="3"/>
-      <c r="L61" s="6"/>
-    </row>
-    <row r="62" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K61" s="6"/>
+    </row>
+    <row r="62" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A62" t="s">
+        <v>201</v>
+      </c>
+      <c r="B62" t="s">
+        <v>202</v>
+      </c>
+      <c r="C62" t="s">
+        <v>203</v>
+      </c>
+      <c r="D62" t="s">
         <v>204</v>
-      </c>
-      <c r="B62" t="s">
-        <v>205</v>
-      </c>
-      <c r="C62" t="s">
-        <v>206</v>
-      </c>
-      <c r="D62" t="s">
-        <v>207</v>
       </c>
       <c r="E62" s="4">
         <v>36</v>
       </c>
       <c r="H62" s="6"/>
       <c r="J62" s="3"/>
-      <c r="L62" s="6"/>
-    </row>
-    <row r="63" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K62" s="6"/>
+    </row>
+    <row r="63" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C63" t="s">
-        <v>208</v>
+        <v>205</v>
       </c>
       <c r="D63" t="s">
-        <v>209</v>
+        <v>206</v>
       </c>
       <c r="E63" s="4">
         <v>18</v>
       </c>
       <c r="H63" s="6"/>
       <c r="J63" s="3"/>
-      <c r="L63" s="6"/>
-    </row>
-    <row r="64" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K63" s="6"/>
+    </row>
+    <row r="64" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C64" t="s">
-        <v>210</v>
+        <v>207</v>
       </c>
       <c r="D64" t="s">
-        <v>211</v>
+        <v>208</v>
       </c>
       <c r="E64" s="4">
         <v>18</v>
       </c>
       <c r="H64" s="6"/>
       <c r="J64" s="3"/>
-      <c r="L64" s="6"/>
-    </row>
-    <row r="65" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K64" s="6"/>
+    </row>
+    <row r="65" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="C65" t="s">
-        <v>212</v>
+        <v>209</v>
       </c>
       <c r="D65" t="s">
-        <v>213</v>
+        <v>210</v>
       </c>
       <c r="E65" s="4">
         <v>13</v>
       </c>
       <c r="H65" s="6"/>
       <c r="J65" s="3"/>
-      <c r="L65" s="6"/>
-    </row>
-    <row r="66" spans="1:12" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K65" s="6"/>
+    </row>
+    <row r="66" spans="1:11" ht="18.75" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A66" t="s">
-        <v>214</v>
+        <v>211</v>
       </c>
       <c r="B66" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="C66" t="s">
-        <v>216</v>
+        <v>213</v>
       </c>
       <c r="D66" t="s">
-        <v>215</v>
+        <v>212</v>
       </c>
       <c r="E66" s="4">
         <v>37</v>
       </c>
       <c r="H66" s="6"/>
       <c r="J66" s="3"/>
-      <c r="L66" s="6"/>
-    </row>
-    <row r="67" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K66" s="6"/>
+    </row>
+    <row r="67" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A67" t="s">
-        <v>217</v>
+        <v>214</v>
       </c>
       <c r="B67" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="C67" t="s">
-        <v>219</v>
+        <v>216</v>
       </c>
       <c r="D67" t="s">
-        <v>218</v>
+        <v>215</v>
       </c>
       <c r="E67" s="4">
         <v>34</v>
       </c>
       <c r="H67" s="6"/>
       <c r="J67" s="3"/>
-      <c r="L67" s="6"/>
-    </row>
-    <row r="68" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K67" s="6"/>
+    </row>
+    <row r="68" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A68" t="s">
-        <v>220</v>
+        <v>217</v>
       </c>
       <c r="B68" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="C68" t="s">
-        <v>222</v>
+        <v>219</v>
       </c>
       <c r="D68" t="s">
-        <v>221</v>
+        <v>218</v>
       </c>
       <c r="E68" s="4">
         <v>38</v>
       </c>
       <c r="H68" s="6"/>
       <c r="J68" s="3"/>
-      <c r="L68" s="6"/>
-    </row>
-    <row r="69" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K68" s="6"/>
+    </row>
+    <row r="69" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="A69" t="s">
-        <v>223</v>
+        <v>220</v>
       </c>
       <c r="B69" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="C69" t="s">
-        <v>225</v>
+        <v>222</v>
       </c>
       <c r="D69" t="s">
-        <v>224</v>
+        <v>221</v>
       </c>
       <c r="E69" s="4">
         <v>27</v>
       </c>
       <c r="H69" s="6"/>
       <c r="J69" s="3"/>
-      <c r="L69" s="6"/>
-    </row>
-    <row r="70" spans="1:12" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
+      <c r="K69" s="6"/>
+    </row>
+    <row r="70" spans="1:11" ht="19.5" hidden="1" customHeight="1" x14ac:dyDescent="0.45">
       <c r="B70" t="s">
-        <v>226</v>
+        <v>223</v>
       </c>
       <c r="E70" s="6"/>
       <c r="H70" s="6"/>
       <c r="J70" s="3"/>
-      <c r="L70" s="6"/>
+      <c r="K70" s="6"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>